<commit_message>
Teacher Activity - Opening Balance
</commit_message>
<xml_diff>
--- a/UMS.UI.Test (OSL)/UMS.UI.Test.ERP/TestData/Teacher/Excel/TeacherActivity.xlsx
+++ b/UMS.UI.Test (OSL)/UMS.UI.Test.ERP/TestData/Teacher/Excel/TeacherActivity.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OPL\source\repos\UMS.UI.Test (OSL)\UMS.UI.Test.ERP\TestData\Teacher\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OPL\source\repos\UMS_Test\UMS.UI.Test (OSL)\UMS.UI.Test.ERP\TestData\Teacher\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{225FC951-BE5C-47AE-8869-AD9059B3C42C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{107F6A72-A136-4EA9-9DD2-FB428D28C6CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,12 +59,6 @@
     <t>12, 10, 0, 14, 58</t>
   </si>
   <si>
-    <t>496  9209 22349   22353 22337  22338</t>
-  </si>
-  <si>
-    <t xml:space="preserve">496, 9209  22349, 22353 </t>
-  </si>
-  <si>
     <t>496 9209 22345 22348 22349 22350 22351 22352 22353</t>
   </si>
   <si>
@@ -72,6 +66,12 @@
   </si>
   <si>
     <t>96, 09, 49, 53, 73, 85</t>
+  </si>
+  <si>
+    <t>496, 9209  22349, 22353 , 22353</t>
+  </si>
+  <si>
+    <t>496  9209 22349   22337 22336</t>
   </si>
 </sst>
 </file>
@@ -475,35 +475,35 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" s="2">
         <v>45771</v>
       </c>
-      <c r="D2" s="8" t="s">
-        <v>12</v>
+      <c r="D2" s="7" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="7" t="s">
-        <v>10</v>
+      <c r="B3" s="6" t="s">
+        <v>8</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>11</v>
+      <c r="D3" s="6" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>8</v>
+      <c r="B4" s="8" t="s">
+        <v>12</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>6</v>

</xml_diff>